<commit_message>
chore(P0-01): xoá hẳn backend nháp cũ services/_deprecated-api-v0
Điều kiện xoá đã đạt từ commit 49f623b: app khách không còn phụ thuộc bản nháp
này nữa. Giữ thêm chỉ tạo chỗ cho người mới đọc nhầm.

Gỡ luôn ba chỗ tài liệu còn trỏ tới nó (README, CLAUDE.md, ghi chú tracker) —
tài liệu trỏ vào thư mục không tồn tại còn khó hiểu hơn là không nhắc gì.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M5wsPS2Wz2e8UfuvEdeSHZ
</commit_message>
<xml_diff>
--- a/docs/GoAn_Project_Tracker.xlsx
+++ b/docs/GoAn_Project_Tracker.xlsx
@@ -2684,11 +2684,11 @@
       <c r="J5" s="59" t="n"/>
       <c r="K5" s="62" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
       <c r="L5" s="64" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="M5" s="63">
         <f>H5*(1-L5)</f>
@@ -2697,7 +2697,7 @@
       <c r="N5" s="62" t="n"/>
       <c r="O5" s="59" t="inlineStr">
         <is>
-          <t>03/09: đã chuyển thành services/_deprecated-api-v0 kèm DEPRECATED.md. Điều kiện xoá ĐÃ ĐẠT (P4-12 xong, app khách không còn phụ thuộc). Chỉ còn thao tác xoá thư mục.</t>
+          <t>03/09 XONG: đã xoá hẳn services/_deprecated-api-v0 khỏi repo sau khi app khách chuyển xong sang API mới (P4-12). Gỡ luôn các chỗ tài liệu còn trỏ tới nó.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: cập nhật tracker và truy vết sau đợt P0-09/P0-11
P0-09 và P0-11 đóng sổ. P0-07 còn 10% là bật branch protection trên giao diện
GitHub — thao tác nằm ngoài repo nên không commit được.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M5wsPS2Wz2e8UfuvEdeSHZ
</commit_message>
<xml_diff>
--- a/docs/GoAn_Project_Tracker.xlsx
+++ b/docs/GoAn_Project_Tracker.xlsx
@@ -2431,16 +2431,16 @@
         </is>
       </c>
       <c r="C24" s="61" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="D24" s="59" t="inlineStr">
         <is>
-          <t>CI 4 job xanh (lint/type/test+ngưỡng độ phủ, alembic check, contract API, build frontend)</t>
+          <t>CI 4 job xanh; secret quản lý bằng SOPS+age có cổng chặn tự động; toàn bộ stack đã chạy thật trên Postgres + Redis + Celery</t>
         </is>
       </c>
       <c r="E24" s="59" t="inlineStr">
         <is>
-          <t>Thiếu: staging, quản lý secret, backup PITR — P0-10/11/18</t>
+          <t>Thiếu: máy chủ staging (P0-10) và backup PITR (P0-18) — cần VPS</t>
         </is>
       </c>
     </row>
@@ -2452,20 +2452,20 @@
       </c>
       <c r="B25" s="60" t="inlineStr">
         <is>
-          <t>Một nửa</t>
+          <t>Gần xong</t>
         </is>
       </c>
       <c r="C25" s="61" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="D25" s="59" t="inlineStr">
         <is>
-          <t>243 test backend xanh, độ phủ 82%; smoke 22 bước và audit 62 lời gọi trên server thật</t>
+          <t>277 test backend + 7 test giao diện Console; smoke 22/22 và audit 76/76 chạy thật trên PostgreSQL</t>
         </is>
       </c>
       <c r="E25" s="59" t="inlineStr">
         <is>
-          <t>Thiếu: test frontend và E2E qua app trên staging</t>
+          <t>Thiếu: E2E qua app trên staging</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       <c r="N11" s="62" t="n"/>
       <c r="O11" s="59" t="inlineStr">
         <is>
-          <t>03/09: CI 4 job. Job Frontend từng đỏ ngay bước cài pnpm (khai version trùng với packageManager) — đã sửa. Còn: bật branch protection trên giao diện GitHub.</t>
+          <t>03/09: CI 5 bước xanh (secret, lint, type, test+độ phủ, money, security) + 3 job khác. Còn: bật branch protection trên giao diện GitHub — thao tác ngoài repo.</t>
         </is>
       </c>
     </row>
@@ -3184,11 +3184,11 @@
       <c r="J13" s="59" t="n"/>
       <c r="K13" s="62" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
       <c r="L13" s="64" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M13" s="63">
         <f>H13*(1-L13)</f>
@@ -3197,7 +3197,7 @@
       <c r="N13" s="62" t="n"/>
       <c r="O13" s="59" t="inlineStr">
         <is>
-          <t>03/09: compose đủ 4 dịch vụ (postgres+postgis, redis, app, worker chạy kèm beat -B); docker compose config hợp lệ. Còn: chạy up kiểm chứng trên máy có Docker.</t>
+          <t>03/09 XONG: chạy thật đủ bộ dịch vụ (Postgres 16 + PostGIS, Redis, uvicorn, celery worker kèm beat). /health + /ready xanh, smoke 22/22, audit 76/76. docker compose config hợp lệ; lệnh `docker compose up` chưa chạy được vì môi trường phiên làm việc không có Docker daemon.</t>
         </is>
       </c>
     </row>
@@ -3304,11 +3304,11 @@
       <c r="J15" s="59" t="n"/>
       <c r="K15" s="62" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã xong</t>
         </is>
       </c>
       <c r="L15" s="64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" s="63">
         <f>H15*(1-L15)</f>
@@ -3317,7 +3317,7 @@
       <c r="N15" s="62" t="n"/>
       <c r="O15" s="59" t="inlineStr">
         <is>
-          <t>Hiện .env đang bị gitignore đúng, nhưng chưa có cơ chế quản lý khoá production</t>
+          <t>03/09 XONG: SOPS + age. .sops.yaml + make secrets-init/new/edit/decrypt/add-key. scripts/check_secrets.py chặn .env chữ thường, khoá riêng và giá trị trông như secret — chạy trong make check và trong CI. Đã thử toàn bộ vòng mã hoá/giải mã.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: tracker ghi nhận P0-10 (70%) và P0-18 (85%) — phần còn lại cần VPS
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M5wsPS2Wz2e8UfuvEdeSHZ
</commit_message>
<xml_diff>
--- a/docs/GoAn_Project_Tracker.xlsx
+++ b/docs/GoAn_Project_Tracker.xlsx
@@ -3248,18 +3248,22 @@
       </c>
       <c r="K14" s="62" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="L14" s="64" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="M14" s="63">
         <f>H14*(1-L14)</f>
         <v/>
       </c>
       <c r="N14" s="62" t="n"/>
-      <c r="O14" s="59" t="n"/>
+      <c r="O14" s="59" t="inlineStr">
+        <is>
+          <t>03/09: deploy/ có đủ docker-compose.prod.yml (api + worker + beat riêng + postgres WAL archiving + redis + Caddy TLS tự động), Caddyfile chặn /metrics ra ngoài, README ghi từng lệnh. CÒN LẠI: mua VPS + trỏ tên miền rồi chạy — phần này nằm ngoài repo.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22.35" customHeight="1" s="38">
       <c r="A15" s="62" t="inlineStr">
@@ -3736,11 +3740,11 @@
       </c>
       <c r="K22" s="62" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="L22" s="64" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="M22" s="63">
         <f>H22*(1-L22)</f>
@@ -3749,7 +3753,7 @@
       <c r="N22" s="62" t="n"/>
       <c r="O22" s="59" t="inlineStr">
         <is>
-          <t>Bắt buộc vì có dữ liệu ký quỹ của tài xế</t>
+          <t>03/09: deploy/backup.sh (dump hằng ngày, tự kiểm bằng pg_restore --list, giữ 30 ngày) + restore.sh + WAL archiving cho PITR. ĐÃ CHẠY THẬT: sao lưu rồi khôi phục sang DB khác, đủ 7 user, 7 chuyến, 5 bút toán ký quỹ, 114 dòng audit. CÒN LẠI: cắm vào máy chủ staging và đặt lịch diễn tập khôi phục mỗi quý.</t>
         </is>
       </c>
     </row>

</xml_diff>